<commit_message>
Daily snapshot: 2026-05-07 23:43 UTC
</commit_message>
<xml_diff>
--- a/data/exports/Aberdeen_Crossing_Availability.xlsx
+++ b/data/exports/Aberdeen_Crossing_Availability.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Availability Matrix" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Availability Matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tier Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Raw Data" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Daily snapshot: 2026-05-08 14:20 UTC
</commit_message>
<xml_diff>
--- a/data/exports/Aberdeen_Crossing_Availability.xlsx
+++ b/data/exports/Aberdeen_Crossing_Availability.xlsx
@@ -475,7 +475,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: aberdeencrossingapts.com/floorplans  |  Snapshot: May 07, 2026  |  Total available units: 75</t>
+          <t>Source: aberdeencrossingapts.com/floorplans  |  Snapshot: May 08, 2026  |  Total available units: 75</t>
         </is>
       </c>
     </row>
@@ -2911,7 +2911,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>23 floor plan types  |  75 available units  |  Snapshot: May 07, 2026</t>
+          <t>23 floor plan types  |  75 available units  |  Snapshot: May 08, 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily snapshot: 2026-05-09 13:56 UTC
</commit_message>
<xml_diff>
--- a/data/exports/Aberdeen_Crossing_Availability.xlsx
+++ b/data/exports/Aberdeen_Crossing_Availability.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G83"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -475,7 +475,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: aberdeencrossingapts.com/floorplans  |  Snapshot: May 08, 2026  |  Total available units: 75</t>
+          <t>Source: aberdeencrossingapts.com/floorplans  |  Snapshot: May 09, 2026  |  Total available units: 73</t>
         </is>
       </c>
     </row>
@@ -519,7 +519,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Studio  (25 available)</t>
+          <t>Studio  (24 available)</t>
         </is>
       </c>
     </row>
@@ -624,12 +624,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tier 02 - Convertible</t>
+          <t>Tier 03 - Studio</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1100-602</t>
+          <t>1100-403</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -638,10 +638,10 @@
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>524</v>
+        <v>468</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>2507</v>
+        <v>2192</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>46113</v>
@@ -660,7 +660,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1100-403</t>
+          <t>1100-503</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -672,7 +672,7 @@
         <v>468</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>2192</v>
+        <v>2217</v>
       </c>
       <c r="G10" s="7" t="n">
         <v>46113</v>
@@ -691,7 +691,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1100-503</t>
+          <t>1100-603</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -703,7 +703,7 @@
         <v>468</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>2217</v>
+        <v>2292</v>
       </c>
       <c r="G11" s="7" t="n">
         <v>46113</v>
@@ -717,12 +717,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Tier 03 - Studio</t>
+          <t>Tier 05 - Convertible</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1100-603</t>
+          <t>1100-205</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -731,10 +731,10 @@
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>468</v>
+        <v>559</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>2292</v>
+        <v>2488</v>
       </c>
       <c r="G12" s="7" t="n">
         <v>46113</v>
@@ -753,7 +753,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1100-205</t>
+          <t>1100-305</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -765,7 +765,7 @@
         <v>559</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>2488</v>
+        <v>2513</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>46113</v>
@@ -784,7 +784,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1100-305</t>
+          <t>1100-405</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -796,7 +796,7 @@
         <v>559</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>2513</v>
+        <v>2563</v>
       </c>
       <c r="G14" s="7" t="n">
         <v>46113</v>
@@ -815,7 +815,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1100-405</t>
+          <t>1100-505</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -827,7 +827,7 @@
         <v>559</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>2563</v>
+        <v>2588</v>
       </c>
       <c r="G15" s="7" t="n">
         <v>46113</v>
@@ -846,7 +846,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1100-505</t>
+          <t>1100-605</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -858,7 +858,7 @@
         <v>559</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>2588</v>
+        <v>2663</v>
       </c>
       <c r="G16" s="7" t="n">
         <v>46113</v>
@@ -872,12 +872,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tier 05 - Convertible</t>
+          <t>Tier 06 - Convertible</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1100-605</t>
+          <t>1100-306</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -886,10 +886,10 @@
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>559</v>
+        <v>539</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>2663</v>
+        <v>2424</v>
       </c>
       <c r="G17" s="7" t="n">
         <v>46113</v>
@@ -908,7 +908,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1100-306</t>
+          <t>1100-406</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -920,7 +920,7 @@
         <v>539</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>2424</v>
+        <v>2449</v>
       </c>
       <c r="G18" s="7" t="n">
         <v>46113</v>
@@ -939,7 +939,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1100-406</t>
+          <t>1100-506</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -951,7 +951,7 @@
         <v>539</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>2449</v>
+        <v>2499</v>
       </c>
       <c r="G19" s="7" t="n">
         <v>46113</v>
@@ -970,7 +970,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1100-506</t>
+          <t>1100-606</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -982,7 +982,7 @@
         <v>539</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>2499</v>
+        <v>2574</v>
       </c>
       <c r="G20" s="7" t="n">
         <v>46113</v>
@@ -996,12 +996,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Tier 06 - Convertible</t>
+          <t>Tier 12 - Convertible</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1100-606</t>
+          <t>1100-312</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1010,10 +1010,10 @@
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>2574</v>
+        <v>2437</v>
       </c>
       <c r="G21" s="7" t="n">
         <v>46113</v>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1100-312</t>
+          <t>1100-412</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1044,7 +1044,7 @@
         <v>542</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>2437</v>
+        <v>2487</v>
       </c>
       <c r="G22" s="7" t="n">
         <v>46113</v>
@@ -1063,7 +1063,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1100-412</t>
+          <t>1100-512</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1075,7 +1075,7 @@
         <v>542</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>2487</v>
+        <v>2512</v>
       </c>
       <c r="G23" s="7" t="n">
         <v>46113</v>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1100-512</t>
+          <t>1100-612</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1106,7 +1106,7 @@
         <v>542</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>2512</v>
+        <v>2587</v>
       </c>
       <c r="G24" s="7" t="n">
         <v>46113</v>
@@ -1120,12 +1120,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Tier 12 - Convertible</t>
+          <t>Tier 13 - Convertible</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1100-612</t>
+          <t>1100-213</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1134,10 +1134,10 @@
         </is>
       </c>
       <c r="E25" s="5" t="n">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>2587</v>
+        <v>2474</v>
       </c>
       <c r="G25" s="7" t="n">
         <v>46113</v>
@@ -1156,7 +1156,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>1100-213</t>
+          <t>1100-313</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1168,7 +1168,7 @@
         <v>539</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>2474</v>
+        <v>2524</v>
       </c>
       <c r="G26" s="7" t="n">
         <v>46113</v>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1100-313</t>
+          <t>1100-413</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1199,7 +1199,7 @@
         <v>539</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>2524</v>
+        <v>2549</v>
       </c>
       <c r="G27" s="7" t="n">
         <v>46113</v>
@@ -1218,7 +1218,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1100-413</t>
+          <t>1100-513</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1230,7 +1230,7 @@
         <v>539</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>2549</v>
+        <v>2574</v>
       </c>
       <c r="G28" s="7" t="n">
         <v>46113</v>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1100-513</t>
+          <t>1100-613</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1261,48 +1261,48 @@
         <v>539</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>2574</v>
+        <v>2649</v>
       </c>
       <c r="G29" s="7" t="n">
         <v>46113</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Studio</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Tier 13 - Convertible</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>1100-613</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>0 / 1</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="n">
-        <v>539</v>
-      </c>
-      <c r="F30" s="6" t="n">
-        <v>2649</v>
-      </c>
-      <c r="G30" s="7" t="n">
-        <v>46113</v>
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>1 Bedroom  (9 available)</t>
+        </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>1 Bedroom  (10 available)</t>
-        </is>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>1 Bedroom</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Tier 02 - Penthouse</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1100-702</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>1 / 1</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>739</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>3761</v>
+      </c>
+      <c r="G31" s="7" t="n">
+        <v>46113</v>
       </c>
     </row>
     <row r="32">
@@ -1313,12 +1313,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Tier 02 - Penthouse</t>
+          <t>Tier 14 - One Bedroom</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>1100-702</t>
+          <t>1100-514</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1327,10 +1327,10 @@
         </is>
       </c>
       <c r="E32" s="5" t="n">
-        <v>739</v>
+        <v>649</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>3761</v>
+        <v>2886</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>46113</v>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1100-414</t>
+          <t>1100-614</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1361,7 +1361,7 @@
         <v>649</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>2861</v>
+        <v>2961</v>
       </c>
       <c r="G33" s="7" t="n">
         <v>46113</v>
@@ -1375,12 +1375,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Tier 14 - One Bedroom</t>
+          <t>Tier 14 - One Bedroom (Terrace)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>1100-514</t>
+          <t>1100-214</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1392,10 +1392,10 @@
         <v>649</v>
       </c>
       <c r="F34" s="6" t="n">
-        <v>2886</v>
+        <v>2856</v>
       </c>
       <c r="G34" s="7" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="35">
@@ -1406,12 +1406,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Tier 14 - One Bedroom</t>
+          <t>Tier 18 - One Bedroom</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>1100-614</t>
+          <t>1100-218</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1420,10 +1420,10 @@
         </is>
       </c>
       <c r="E35" s="5" t="n">
-        <v>649</v>
+        <v>656</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>2961</v>
+        <v>2690</v>
       </c>
       <c r="G35" s="7" t="n">
         <v>46113</v>
@@ -1437,12 +1437,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Tier 14 - One Bedroom (Terrace)</t>
+          <t>Tier 18 - One Bedroom</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>1100-214</t>
+          <t>1100-318</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1451,13 +1451,13 @@
         </is>
       </c>
       <c r="E36" s="5" t="n">
-        <v>649</v>
+        <v>656</v>
       </c>
       <c r="F36" s="6" t="n">
-        <v>2856</v>
+        <v>2715</v>
       </c>
       <c r="G36" s="7" t="n">
-        <v>46143</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="37">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>1100-218</t>
+          <t>1100-418</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1485,10 +1485,10 @@
         <v>656</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>2690</v>
+        <v>2740</v>
       </c>
       <c r="G37" s="7" t="n">
-        <v>46113</v>
+        <v>46135</v>
       </c>
     </row>
     <row r="38">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>1100-318</t>
+          <t>1100-518</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1516,7 +1516,7 @@
         <v>656</v>
       </c>
       <c r="F38" s="6" t="n">
-        <v>2715</v>
+        <v>2765</v>
       </c>
       <c r="G38" s="7" t="n">
         <v>46113</v>
@@ -1530,12 +1530,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Tier 18 - One Bedroom</t>
+          <t>Tier 18 - Penthouse</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>1100-418</t>
+          <t>1100-718</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1547,79 +1547,79 @@
         <v>656</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>2740</v>
+        <v>3375</v>
       </c>
       <c r="G39" s="7" t="n">
-        <v>46135</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>1 Bedroom</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Tier 18 - One Bedroom</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>1100-518</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>1 / 1</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="n">
-        <v>656</v>
-      </c>
-      <c r="F40" s="6" t="n">
-        <v>2765</v>
-      </c>
-      <c r="G40" s="7" t="n">
-        <v>46113</v>
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>2 Bedroom  (30 available)</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1 Bedroom</t>
+          <t>2 Bedroom</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Tier 18 - Penthouse</t>
+          <t>Tier 01 - Penthouse</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>1100-718</t>
+          <t>1100-701</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>1 / 1</t>
+          <t>2 / 2</t>
         </is>
       </c>
       <c r="E41" s="5" t="n">
-        <v>656</v>
+        <v>975</v>
       </c>
       <c r="F41" s="6" t="n">
-        <v>3375</v>
+        <v>4534</v>
       </c>
       <c r="G41" s="7" t="n">
         <v>46113</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>2 Bedroom  (30 available)</t>
-        </is>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2 Bedroom</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Tier 01 - Two Bedroom</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1100-201</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2 / 2</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="n">
+        <v>975</v>
+      </c>
+      <c r="F42" s="6" t="n">
+        <v>3910</v>
+      </c>
+      <c r="G42" s="7" t="n">
+        <v>46113</v>
       </c>
     </row>
     <row r="43">
@@ -1630,12 +1630,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Tier 01 - Penthouse</t>
+          <t>Tier 01 - Two Bedroom</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>1100-701</t>
+          <t>1100-501</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1647,7 +1647,7 @@
         <v>975</v>
       </c>
       <c r="F43" s="6" t="n">
-        <v>4534</v>
+        <v>4010</v>
       </c>
       <c r="G43" s="7" t="n">
         <v>46113</v>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>1100-201</t>
+          <t>1100-601</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1678,7 +1678,7 @@
         <v>975</v>
       </c>
       <c r="F44" s="6" t="n">
-        <v>3910</v>
+        <v>4085</v>
       </c>
       <c r="G44" s="7" t="n">
         <v>46113</v>
@@ -1692,12 +1692,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Tier 01 - Two Bedroom</t>
+          <t>Tier 04 - Two Bedroom</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>1100-501</t>
+          <t>1100-304</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1706,10 +1706,10 @@
         </is>
       </c>
       <c r="E45" s="5" t="n">
-        <v>975</v>
+        <v>990</v>
       </c>
       <c r="F45" s="6" t="n">
-        <v>4010</v>
+        <v>3970</v>
       </c>
       <c r="G45" s="7" t="n">
         <v>46113</v>
@@ -1723,12 +1723,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Tier 01 - Two Bedroom</t>
+          <t>Tier 04 - Two Bedroom</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>1100-601</t>
+          <t>1100-404</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1737,10 +1737,10 @@
         </is>
       </c>
       <c r="E46" s="5" t="n">
-        <v>975</v>
+        <v>990</v>
       </c>
       <c r="F46" s="6" t="n">
-        <v>4085</v>
+        <v>4045</v>
       </c>
       <c r="G46" s="7" t="n">
         <v>46113</v>
@@ -1759,7 +1759,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>1100-304</t>
+          <t>1100-504</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1771,7 +1771,7 @@
         <v>990</v>
       </c>
       <c r="F47" s="6" t="n">
-        <v>3970</v>
+        <v>4070</v>
       </c>
       <c r="G47" s="7" t="n">
         <v>46113</v>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>1100-404</t>
+          <t>1100-604</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1802,7 +1802,7 @@
         <v>990</v>
       </c>
       <c r="F48" s="6" t="n">
-        <v>4045</v>
+        <v>4145</v>
       </c>
       <c r="G48" s="7" t="n">
         <v>46113</v>
@@ -1816,12 +1816,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Tier 04 - Two Bedroom</t>
+          <t>Tier 08 - Two Bedroom</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>1100-504</t>
+          <t>1100-208</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1830,10 +1830,10 @@
         </is>
       </c>
       <c r="E49" s="5" t="n">
-        <v>990</v>
+        <v>982</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>4070</v>
+        <v>3943</v>
       </c>
       <c r="G49" s="7" t="n">
         <v>46113</v>
@@ -1847,12 +1847,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Tier 04 - Two Bedroom</t>
+          <t>Tier 08 - Two Bedroom</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>1100-604</t>
+          <t>1100-308</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1861,10 +1861,10 @@
         </is>
       </c>
       <c r="E50" s="5" t="n">
-        <v>990</v>
+        <v>982</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>4145</v>
+        <v>3993</v>
       </c>
       <c r="G50" s="7" t="n">
         <v>46113</v>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>1100-208</t>
+          <t>1100-408</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1895,7 +1895,7 @@
         <v>982</v>
       </c>
       <c r="F51" s="6" t="n">
-        <v>3943</v>
+        <v>4018</v>
       </c>
       <c r="G51" s="7" t="n">
         <v>46113</v>
@@ -1914,7 +1914,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>1100-308</t>
+          <t>1100-508</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1926,7 +1926,7 @@
         <v>982</v>
       </c>
       <c r="F52" s="6" t="n">
-        <v>3993</v>
+        <v>4043</v>
       </c>
       <c r="G52" s="7" t="n">
         <v>46113</v>
@@ -1945,7 +1945,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>1100-408</t>
+          <t>1100-608</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1957,7 +1957,7 @@
         <v>982</v>
       </c>
       <c r="F53" s="6" t="n">
-        <v>4018</v>
+        <v>4118</v>
       </c>
       <c r="G53" s="7" t="n">
         <v>46113</v>
@@ -1971,12 +1971,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Tier 08 - Two Bedroom</t>
+          <t>Tier 10 - Two Bedroom</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>1100-508</t>
+          <t>1100-310</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1985,13 +1985,13 @@
         </is>
       </c>
       <c r="E54" s="5" t="n">
-        <v>982</v>
+        <v>934</v>
       </c>
       <c r="F54" s="6" t="n">
-        <v>4043</v>
+        <v>3745</v>
       </c>
       <c r="G54" s="7" t="n">
-        <v>46113</v>
+        <v>46094</v>
       </c>
     </row>
     <row r="55">
@@ -2002,12 +2002,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Tier 08 - Two Bedroom</t>
+          <t>Tier 10 - Two Bedroom</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>1100-608</t>
+          <t>1100-410</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2016,10 +2016,10 @@
         </is>
       </c>
       <c r="E55" s="5" t="n">
-        <v>982</v>
+        <v>934</v>
       </c>
       <c r="F55" s="6" t="n">
-        <v>4118</v>
+        <v>3820</v>
       </c>
       <c r="G55" s="7" t="n">
         <v>46113</v>
@@ -2038,7 +2038,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>1100-310</t>
+          <t>1100-610</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2050,10 +2050,10 @@
         <v>934</v>
       </c>
       <c r="F56" s="6" t="n">
-        <v>3745</v>
+        <v>3920</v>
       </c>
       <c r="G56" s="7" t="n">
-        <v>46094</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="57">
@@ -2064,12 +2064,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Tier 10 - Two Bedroom</t>
+          <t>Tier 10 - Two Bedroom (Terrace)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>1100-410</t>
+          <t>1100-210</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2081,7 +2081,7 @@
         <v>934</v>
       </c>
       <c r="F57" s="6" t="n">
-        <v>3820</v>
+        <v>4203</v>
       </c>
       <c r="G57" s="7" t="n">
         <v>46113</v>
@@ -2095,12 +2095,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Tier 10 - Two Bedroom</t>
+          <t>Tier 11 - Two Bedroom</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>1100-610</t>
+          <t>1100-311</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2109,10 +2109,10 @@
         </is>
       </c>
       <c r="E58" s="5" t="n">
-        <v>934</v>
+        <v>972</v>
       </c>
       <c r="F58" s="6" t="n">
-        <v>3920</v>
+        <v>3898</v>
       </c>
       <c r="G58" s="7" t="n">
         <v>46113</v>
@@ -2126,12 +2126,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Tier 10 - Two Bedroom (Terrace)</t>
+          <t>Tier 11 - Two Bedroom</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>1100-210</t>
+          <t>1100-411</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2140,10 +2140,10 @@
         </is>
       </c>
       <c r="E59" s="5" t="n">
-        <v>934</v>
+        <v>972</v>
       </c>
       <c r="F59" s="6" t="n">
-        <v>4203</v>
+        <v>3973</v>
       </c>
       <c r="G59" s="7" t="n">
         <v>46113</v>
@@ -2162,7 +2162,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>1100-311</t>
+          <t>1100-511</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2174,7 +2174,7 @@
         <v>972</v>
       </c>
       <c r="F60" s="6" t="n">
-        <v>3898</v>
+        <v>3998</v>
       </c>
       <c r="G60" s="7" t="n">
         <v>46113</v>
@@ -2193,7 +2193,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>1100-411</t>
+          <t>1100-611</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2202,10 +2202,10 @@
         </is>
       </c>
       <c r="E61" s="5" t="n">
-        <v>972</v>
+        <v>892</v>
       </c>
       <c r="F61" s="6" t="n">
-        <v>3973</v>
+        <v>3732</v>
       </c>
       <c r="G61" s="7" t="n">
         <v>46113</v>
@@ -2219,12 +2219,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Tier 11 - Two Bedroom</t>
+          <t>Tier 15 - Two Bedroom</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>1100-511</t>
+          <t>1100-215</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2233,10 +2233,10 @@
         </is>
       </c>
       <c r="E62" s="5" t="n">
-        <v>972</v>
+        <v>1028</v>
       </c>
       <c r="F62" s="6" t="n">
-        <v>3998</v>
+        <v>4133</v>
       </c>
       <c r="G62" s="7" t="n">
         <v>46113</v>
@@ -2250,12 +2250,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Tier 11 - Two Bedroom</t>
+          <t>Tier 15 - Two Bedroom</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>1100-611</t>
+          <t>1100-315</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2264,10 +2264,10 @@
         </is>
       </c>
       <c r="E63" s="5" t="n">
-        <v>892</v>
+        <v>1028</v>
       </c>
       <c r="F63" s="6" t="n">
-        <v>3732</v>
+        <v>4183</v>
       </c>
       <c r="G63" s="7" t="n">
         <v>46113</v>
@@ -2286,7 +2286,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>1100-215</t>
+          <t>1100-415</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2298,7 +2298,7 @@
         <v>1028</v>
       </c>
       <c r="F64" s="6" t="n">
-        <v>4133</v>
+        <v>4233</v>
       </c>
       <c r="G64" s="7" t="n">
         <v>46113</v>
@@ -2317,7 +2317,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>1100-315</t>
+          <t>1100-515</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2329,7 +2329,7 @@
         <v>1028</v>
       </c>
       <c r="F65" s="6" t="n">
-        <v>4183</v>
+        <v>4233</v>
       </c>
       <c r="G65" s="7" t="n">
         <v>46113</v>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>1100-415</t>
+          <t>1100-615</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2360,7 +2360,7 @@
         <v>1028</v>
       </c>
       <c r="F66" s="6" t="n">
-        <v>4233</v>
+        <v>4308</v>
       </c>
       <c r="G66" s="7" t="n">
         <v>46113</v>
@@ -2374,12 +2374,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Tier 15 - Two Bedroom</t>
+          <t>Tier 17 - Two Bedroom</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>1100-515</t>
+          <t>1100-217</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2388,10 +2388,10 @@
         </is>
       </c>
       <c r="E67" s="5" t="n">
-        <v>1028</v>
+        <v>917</v>
       </c>
       <c r="F67" s="6" t="n">
-        <v>4233</v>
+        <v>3495</v>
       </c>
       <c r="G67" s="7" t="n">
         <v>46113</v>
@@ -2405,12 +2405,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Tier 15 - Two Bedroom</t>
+          <t>Tier 17 - Two Bedroom</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>1100-615</t>
+          <t>1100-317</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2419,10 +2419,10 @@
         </is>
       </c>
       <c r="E68" s="5" t="n">
-        <v>1028</v>
+        <v>917</v>
       </c>
       <c r="F68" s="6" t="n">
-        <v>4308</v>
+        <v>3721</v>
       </c>
       <c r="G68" s="7" t="n">
         <v>46113</v>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>1100-217</t>
+          <t>1100-517</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2453,7 +2453,7 @@
         <v>917</v>
       </c>
       <c r="F69" s="6" t="n">
-        <v>3495</v>
+        <v>3771</v>
       </c>
       <c r="G69" s="7" t="n">
         <v>46113</v>
@@ -2472,7 +2472,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>1100-317</t>
+          <t>1100-617</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2484,79 +2484,79 @@
         <v>917</v>
       </c>
       <c r="F70" s="6" t="n">
-        <v>3721</v>
+        <v>3846</v>
       </c>
       <c r="G70" s="7" t="n">
         <v>46113</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>2 Bedroom</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Tier 17 - Two Bedroom</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>1100-517</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>2 / 2</t>
-        </is>
-      </c>
-      <c r="E71" s="5" t="n">
-        <v>917</v>
-      </c>
-      <c r="F71" s="6" t="n">
-        <v>3771</v>
-      </c>
-      <c r="G71" s="7" t="n">
-        <v>46113</v>
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>3 Bedroom  (10 available)</t>
+        </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2 Bedroom</t>
+          <t>3 Bedroom</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Tier 17 - Two Bedroom</t>
+          <t>Tier 07 - Three Bedroom</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>1100-617</t>
+          <t>1100-307</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>2 / 2</t>
+          <t>3 / 2</t>
         </is>
       </c>
       <c r="E72" s="5" t="n">
-        <v>917</v>
+        <v>1166</v>
       </c>
       <c r="F72" s="6" t="n">
-        <v>3846</v>
+        <v>4964</v>
       </c>
       <c r="G72" s="7" t="n">
         <v>46113</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="4" t="inlineStr">
-        <is>
-          <t>3 Bedroom  (10 available)</t>
-        </is>
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>3 Bedroom</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Tier 07 - Three Bedroom</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>1100-407</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>3 / 2</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="n">
+        <v>1166</v>
+      </c>
+      <c r="F73" s="6" t="n">
+        <v>4989</v>
+      </c>
+      <c r="G73" s="7" t="n">
+        <v>46113</v>
       </c>
     </row>
     <row r="74">
@@ -2572,7 +2572,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>1100-307</t>
+          <t>1100-507</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2584,7 +2584,7 @@
         <v>1166</v>
       </c>
       <c r="F74" s="6" t="n">
-        <v>4964</v>
+        <v>5014</v>
       </c>
       <c r="G74" s="7" t="n">
         <v>46113</v>
@@ -2603,7 +2603,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>1100-407</t>
+          <t>1100-607</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2615,7 +2615,7 @@
         <v>1166</v>
       </c>
       <c r="F75" s="6" t="n">
-        <v>4989</v>
+        <v>5089</v>
       </c>
       <c r="G75" s="7" t="n">
         <v>46113</v>
@@ -2629,12 +2629,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Tier 07 - Three Bedroom</t>
+          <t>Tier 19 - Penthouse</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>1100-507</t>
+          <t>1100-719</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2643,10 +2643,10 @@
         </is>
       </c>
       <c r="E76" s="5" t="n">
-        <v>1166</v>
+        <v>1327</v>
       </c>
       <c r="F76" s="6" t="n">
-        <v>5014</v>
+        <v>6696</v>
       </c>
       <c r="G76" s="7" t="n">
         <v>46113</v>
@@ -2660,12 +2660,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Tier 07 - Three Bedroom</t>
+          <t>Tier 19 - Three Bedroom</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>1100-607</t>
+          <t>1100-219</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2674,10 +2674,10 @@
         </is>
       </c>
       <c r="E77" s="5" t="n">
-        <v>1166</v>
+        <v>1327</v>
       </c>
       <c r="F77" s="6" t="n">
-        <v>5089</v>
+        <v>5582</v>
       </c>
       <c r="G77" s="7" t="n">
         <v>46113</v>
@@ -2691,12 +2691,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Tier 19 - Penthouse</t>
+          <t>Tier 19 - Three Bedroom</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>1100-719</t>
+          <t>1100-319</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2708,7 +2708,7 @@
         <v>1327</v>
       </c>
       <c r="F78" s="6" t="n">
-        <v>6696</v>
+        <v>5607</v>
       </c>
       <c r="G78" s="7" t="n">
         <v>46113</v>
@@ -2727,7 +2727,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>1100-219</t>
+          <t>1100-419</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2739,7 +2739,7 @@
         <v>1327</v>
       </c>
       <c r="F79" s="6" t="n">
-        <v>5582</v>
+        <v>5632</v>
       </c>
       <c r="G79" s="7" t="n">
         <v>46113</v>
@@ -2758,7 +2758,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>1100-319</t>
+          <t>1100-519</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2770,7 +2770,7 @@
         <v>1327</v>
       </c>
       <c r="F80" s="6" t="n">
-        <v>5607</v>
+        <v>5657</v>
       </c>
       <c r="G80" s="7" t="n">
         <v>46113</v>
@@ -2789,7 +2789,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>1100-419</t>
+          <t>1100-619</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2801,71 +2801,9 @@
         <v>1327</v>
       </c>
       <c r="F81" s="6" t="n">
-        <v>5632</v>
+        <v>5732</v>
       </c>
       <c r="G81" s="7" t="n">
-        <v>46113</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>3 Bedroom</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>Tier 19 - Three Bedroom</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>1100-519</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>3 / 2</t>
-        </is>
-      </c>
-      <c r="E82" s="5" t="n">
-        <v>1327</v>
-      </c>
-      <c r="F82" s="6" t="n">
-        <v>5657</v>
-      </c>
-      <c r="G82" s="7" t="n">
-        <v>46113</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>3 Bedroom</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>Tier 19 - Three Bedroom</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>1100-619</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>3 / 2</t>
-        </is>
-      </c>
-      <c r="E83" s="5" t="n">
-        <v>1327</v>
-      </c>
-      <c r="F83" s="6" t="n">
-        <v>5732</v>
-      </c>
-      <c r="G83" s="7" t="n">
         <v>46113</v>
       </c>
     </row>
@@ -2873,9 +2811,9 @@
   <mergeCells count="6">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="A42:G42"/>
-    <mergeCell ref="A73:G73"/>
+    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A71:G71"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2911,7 +2849,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>23 floor plan types  |  75 available units  |  Snapshot: May 08, 2026</t>
+          <t>23 floor plan types  |  73 available units  |  Snapshot: May 09, 2026</t>
         </is>
       </c>
     </row>
@@ -2979,11 +2917,11 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>$2,332 – $2,507</t>
+          <t>$2,332 – $2,432</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>46113</v>
@@ -3203,11 +3141,11 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>$2,861 – $2,961</t>
+          <t>$2,886 – $2,961</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>46113</v>
@@ -3719,7 +3657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3906,12 +3844,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1100-602</t>
+          <t>1100-403</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tier 02 - Convertible</t>
+          <t>Tier 03 - Studio</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3926,13 +3864,13 @@
         <v>1</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>524</v>
+        <v>468</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>2507</v>
+        <v>2192</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>2507</v>
+        <v>2192</v>
       </c>
       <c r="I5" s="7" t="n">
         <v>46113</v>
@@ -3945,7 +3883,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1100-403</t>
+          <t>1100-503</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3968,10 +3906,10 @@
         <v>468</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>2192</v>
+        <v>2217</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>2192</v>
+        <v>2217</v>
       </c>
       <c r="I6" s="7" t="n">
         <v>46113</v>
@@ -3984,7 +3922,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1100-503</t>
+          <t>1100-603</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4007,10 +3945,10 @@
         <v>468</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>2217</v>
+        <v>2292</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>2217</v>
+        <v>2292</v>
       </c>
       <c r="I7" s="7" t="n">
         <v>46113</v>
@@ -4023,12 +3961,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1100-603</t>
+          <t>1100-205</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tier 03 - Studio</t>
+          <t>Tier 05 - Convertible</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -4043,13 +3981,13 @@
         <v>1</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>468</v>
+        <v>559</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>2292</v>
+        <v>2488</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>2292</v>
+        <v>2488</v>
       </c>
       <c r="I8" s="7" t="n">
         <v>46113</v>
@@ -4062,7 +4000,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1100-205</t>
+          <t>1100-305</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4085,10 +4023,10 @@
         <v>559</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>2488</v>
+        <v>2513</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>2488</v>
+        <v>2513</v>
       </c>
       <c r="I9" s="7" t="n">
         <v>46113</v>
@@ -4101,7 +4039,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1100-305</t>
+          <t>1100-405</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4124,10 +4062,10 @@
         <v>559</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>2513</v>
+        <v>2563</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>2513</v>
+        <v>2563</v>
       </c>
       <c r="I10" s="7" t="n">
         <v>46113</v>
@@ -4140,7 +4078,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1100-405</t>
+          <t>1100-505</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4163,10 +4101,10 @@
         <v>559</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>2563</v>
+        <v>2588</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>2563</v>
+        <v>2588</v>
       </c>
       <c r="I11" s="7" t="n">
         <v>46113</v>
@@ -4179,7 +4117,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1100-505</t>
+          <t>1100-605</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4202,10 +4140,10 @@
         <v>559</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>2588</v>
+        <v>2663</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>2588</v>
+        <v>2663</v>
       </c>
       <c r="I12" s="7" t="n">
         <v>46113</v>
@@ -4218,12 +4156,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1100-605</t>
+          <t>1100-306</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Tier 05 - Convertible</t>
+          <t>Tier 06 - Convertible</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -4238,13 +4176,13 @@
         <v>1</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>559</v>
+        <v>539</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>2663</v>
+        <v>2424</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>2663</v>
+        <v>2424</v>
       </c>
       <c r="I13" s="7" t="n">
         <v>46113</v>
@@ -4257,7 +4195,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1100-306</t>
+          <t>1100-406</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -4280,10 +4218,10 @@
         <v>539</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>2424</v>
+        <v>2449</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>2424</v>
+        <v>2449</v>
       </c>
       <c r="I14" s="7" t="n">
         <v>46113</v>
@@ -4296,7 +4234,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1100-406</t>
+          <t>1100-506</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -4319,10 +4257,10 @@
         <v>539</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>2449</v>
+        <v>2499</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>2449</v>
+        <v>2499</v>
       </c>
       <c r="I15" s="7" t="n">
         <v>46113</v>
@@ -4335,7 +4273,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1100-506</t>
+          <t>1100-606</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -4358,10 +4296,10 @@
         <v>539</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>2499</v>
+        <v>2574</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>2499</v>
+        <v>2574</v>
       </c>
       <c r="I16" s="7" t="n">
         <v>46113</v>
@@ -4374,12 +4312,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1100-606</t>
+          <t>1100-312</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tier 06 - Convertible</t>
+          <t>Tier 12 - Convertible</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -4394,13 +4332,13 @@
         <v>1</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>2574</v>
+        <v>2437</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>2574</v>
+        <v>2437</v>
       </c>
       <c r="I17" s="7" t="n">
         <v>46113</v>
@@ -4413,7 +4351,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1100-312</t>
+          <t>1100-412</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -4436,10 +4374,10 @@
         <v>542</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>2437</v>
+        <v>2487</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>2437</v>
+        <v>2487</v>
       </c>
       <c r="I18" s="7" t="n">
         <v>46113</v>
@@ -4452,7 +4390,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1100-412</t>
+          <t>1100-512</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -4475,10 +4413,10 @@
         <v>542</v>
       </c>
       <c r="G19" s="6" t="n">
-        <v>2487</v>
+        <v>2512</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>2487</v>
+        <v>2512</v>
       </c>
       <c r="I19" s="7" t="n">
         <v>46113</v>
@@ -4491,7 +4429,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1100-512</t>
+          <t>1100-612</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -4514,10 +4452,10 @@
         <v>542</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>2512</v>
+        <v>2587</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>2512</v>
+        <v>2587</v>
       </c>
       <c r="I20" s="7" t="n">
         <v>46113</v>
@@ -4530,12 +4468,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1100-612</t>
+          <t>1100-213</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Tier 12 - Convertible</t>
+          <t>Tier 13 - Convertible</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -4550,13 +4488,13 @@
         <v>1</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>2587</v>
+        <v>2474</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>2587</v>
+        <v>2474</v>
       </c>
       <c r="I21" s="7" t="n">
         <v>46113</v>
@@ -4569,7 +4507,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1100-213</t>
+          <t>1100-313</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -4592,10 +4530,10 @@
         <v>539</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>2474</v>
+        <v>2524</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>2474</v>
+        <v>2524</v>
       </c>
       <c r="I22" s="7" t="n">
         <v>46113</v>
@@ -4608,7 +4546,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1100-313</t>
+          <t>1100-413</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4631,10 +4569,10 @@
         <v>539</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>2524</v>
+        <v>2549</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>2524</v>
+        <v>2549</v>
       </c>
       <c r="I23" s="7" t="n">
         <v>46113</v>
@@ -4647,7 +4585,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1100-413</t>
+          <t>1100-513</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4670,10 +4608,10 @@
         <v>539</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>2549</v>
+        <v>2574</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>2549</v>
+        <v>2574</v>
       </c>
       <c r="I24" s="7" t="n">
         <v>46113</v>
@@ -4686,7 +4624,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1100-513</t>
+          <t>1100-613</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4709,10 +4647,10 @@
         <v>539</v>
       </c>
       <c r="G25" s="6" t="n">
-        <v>2574</v>
+        <v>2649</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>2574</v>
+        <v>2649</v>
       </c>
       <c r="I25" s="7" t="n">
         <v>46113</v>
@@ -4725,33 +4663,33 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1100-613</t>
+          <t>1100-702</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Tier 13 - Convertible</t>
+          <t>Tier 02 - Penthouse</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Studio</t>
+          <t>1 Bedroom</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E26" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>539</v>
+        <v>739</v>
       </c>
       <c r="G26" s="6" t="n">
-        <v>2649</v>
+        <v>3761</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>2649</v>
+        <v>3761</v>
       </c>
       <c r="I26" s="7" t="n">
         <v>46113</v>
@@ -4764,12 +4702,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1100-702</t>
+          <t>1100-514</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Tier 02 - Penthouse</t>
+          <t>Tier 14 - One Bedroom</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -4784,13 +4722,13 @@
         <v>1</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>739</v>
+        <v>649</v>
       </c>
       <c r="G27" s="6" t="n">
-        <v>3761</v>
+        <v>2886</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>3761</v>
+        <v>2886</v>
       </c>
       <c r="I27" s="7" t="n">
         <v>46113</v>
@@ -4803,7 +4741,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1100-414</t>
+          <t>1100-614</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -4826,10 +4764,10 @@
         <v>649</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>2861</v>
+        <v>2961</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>2861</v>
+        <v>2961</v>
       </c>
       <c r="I28" s="7" t="n">
         <v>46113</v>
@@ -4842,12 +4780,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1100-514</t>
+          <t>1100-214</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Tier 14 - One Bedroom</t>
+          <t>Tier 14 - One Bedroom (Terrace)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -4865,13 +4803,13 @@
         <v>649</v>
       </c>
       <c r="G29" s="6" t="n">
-        <v>2886</v>
+        <v>2856</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>2886</v>
+        <v>2856</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="J29" s="8">
         <f>G29/F29</f>
@@ -4881,12 +4819,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1100-614</t>
+          <t>1100-218</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Tier 14 - One Bedroom</t>
+          <t>Tier 18 - One Bedroom</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -4901,13 +4839,13 @@
         <v>1</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>649</v>
+        <v>656</v>
       </c>
       <c r="G30" s="6" t="n">
-        <v>2961</v>
+        <v>2690</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>2961</v>
+        <v>2690</v>
       </c>
       <c r="I30" s="7" t="n">
         <v>46113</v>
@@ -4920,12 +4858,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1100-214</t>
+          <t>1100-318</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Tier 14 - One Bedroom (Terrace)</t>
+          <t>Tier 18 - One Bedroom</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -4940,16 +4878,16 @@
         <v>1</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>649</v>
+        <v>656</v>
       </c>
       <c r="G31" s="6" t="n">
-        <v>2856</v>
+        <v>2715</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>2856</v>
+        <v>2715</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>46143</v>
+        <v>46113</v>
       </c>
       <c r="J31" s="8">
         <f>G31/F31</f>
@@ -4959,7 +4897,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1100-218</t>
+          <t>1100-418</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -4982,13 +4920,13 @@
         <v>656</v>
       </c>
       <c r="G32" s="6" t="n">
-        <v>2690</v>
+        <v>2740</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>2690</v>
+        <v>2740</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>46113</v>
+        <v>46135</v>
       </c>
       <c r="J32" s="8">
         <f>G32/F32</f>
@@ -4998,7 +4936,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1100-318</t>
+          <t>1100-518</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -5021,10 +4959,10 @@
         <v>656</v>
       </c>
       <c r="G33" s="6" t="n">
-        <v>2715</v>
+        <v>2765</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>2715</v>
+        <v>2765</v>
       </c>
       <c r="I33" s="7" t="n">
         <v>46113</v>
@@ -5037,12 +4975,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1100-418</t>
+          <t>1100-718</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Tier 18 - One Bedroom</t>
+          <t>Tier 18 - Penthouse</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -5060,13 +4998,13 @@
         <v>656</v>
       </c>
       <c r="G34" s="6" t="n">
-        <v>2740</v>
+        <v>3375</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>2740</v>
+        <v>3375</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>46135</v>
+        <v>46113</v>
       </c>
       <c r="J34" s="8">
         <f>G34/F34</f>
@@ -5076,33 +5014,33 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1100-518</t>
+          <t>1100-701</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Tier 18 - One Bedroom</t>
+          <t>Tier 01 - Penthouse</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>1 Bedroom</t>
+          <t>2 Bedroom</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F35" s="5" t="n">
-        <v>656</v>
+        <v>975</v>
       </c>
       <c r="G35" s="6" t="n">
-        <v>2765</v>
+        <v>4534</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>2765</v>
+        <v>4534</v>
       </c>
       <c r="I35" s="7" t="n">
         <v>46113</v>
@@ -5115,33 +5053,33 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1100-718</t>
+          <t>1100-201</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Tier 18 - Penthouse</t>
+          <t>Tier 01 - Two Bedroom</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>1 Bedroom</t>
+          <t>2 Bedroom</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F36" s="5" t="n">
-        <v>656</v>
+        <v>975</v>
       </c>
       <c r="G36" s="6" t="n">
-        <v>3375</v>
+        <v>3910</v>
       </c>
       <c r="H36" s="6" t="n">
-        <v>3375</v>
+        <v>3910</v>
       </c>
       <c r="I36" s="7" t="n">
         <v>46113</v>
@@ -5154,12 +5092,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1100-701</t>
+          <t>1100-501</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Tier 01 - Penthouse</t>
+          <t>Tier 01 - Two Bedroom</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -5177,10 +5115,10 @@
         <v>975</v>
       </c>
       <c r="G37" s="6" t="n">
-        <v>4534</v>
+        <v>4010</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>4534</v>
+        <v>4010</v>
       </c>
       <c r="I37" s="7" t="n">
         <v>46113</v>
@@ -5193,7 +5131,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1100-201</t>
+          <t>1100-601</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -5216,10 +5154,10 @@
         <v>975</v>
       </c>
       <c r="G38" s="6" t="n">
-        <v>3910</v>
+        <v>4085</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>3910</v>
+        <v>4085</v>
       </c>
       <c r="I38" s="7" t="n">
         <v>46113</v>
@@ -5232,12 +5170,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1100-501</t>
+          <t>1100-304</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Tier 01 - Two Bedroom</t>
+          <t>Tier 04 - Two Bedroom</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -5252,13 +5190,13 @@
         <v>2</v>
       </c>
       <c r="F39" s="5" t="n">
-        <v>975</v>
+        <v>990</v>
       </c>
       <c r="G39" s="6" t="n">
-        <v>4010</v>
+        <v>3970</v>
       </c>
       <c r="H39" s="6" t="n">
-        <v>4010</v>
+        <v>3970</v>
       </c>
       <c r="I39" s="7" t="n">
         <v>46113</v>
@@ -5271,12 +5209,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1100-601</t>
+          <t>1100-404</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Tier 01 - Two Bedroom</t>
+          <t>Tier 04 - Two Bedroom</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -5291,13 +5229,13 @@
         <v>2</v>
       </c>
       <c r="F40" s="5" t="n">
-        <v>975</v>
+        <v>990</v>
       </c>
       <c r="G40" s="6" t="n">
-        <v>4085</v>
+        <v>4045</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>4085</v>
+        <v>4045</v>
       </c>
       <c r="I40" s="7" t="n">
         <v>46113</v>
@@ -5310,7 +5248,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1100-304</t>
+          <t>1100-504</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -5333,10 +5271,10 @@
         <v>990</v>
       </c>
       <c r="G41" s="6" t="n">
-        <v>3970</v>
+        <v>4070</v>
       </c>
       <c r="H41" s="6" t="n">
-        <v>3970</v>
+        <v>4070</v>
       </c>
       <c r="I41" s="7" t="n">
         <v>46113</v>
@@ -5349,7 +5287,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1100-404</t>
+          <t>1100-604</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -5372,10 +5310,10 @@
         <v>990</v>
       </c>
       <c r="G42" s="6" t="n">
-        <v>4045</v>
+        <v>4145</v>
       </c>
       <c r="H42" s="6" t="n">
-        <v>4045</v>
+        <v>4145</v>
       </c>
       <c r="I42" s="7" t="n">
         <v>46113</v>
@@ -5388,12 +5326,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1100-504</t>
+          <t>1100-208</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Tier 04 - Two Bedroom</t>
+          <t>Tier 08 - Two Bedroom</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -5408,13 +5346,13 @@
         <v>2</v>
       </c>
       <c r="F43" s="5" t="n">
-        <v>990</v>
+        <v>982</v>
       </c>
       <c r="G43" s="6" t="n">
-        <v>4070</v>
+        <v>3943</v>
       </c>
       <c r="H43" s="6" t="n">
-        <v>4070</v>
+        <v>3943</v>
       </c>
       <c r="I43" s="7" t="n">
         <v>46113</v>
@@ -5427,12 +5365,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1100-604</t>
+          <t>1100-308</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Tier 04 - Two Bedroom</t>
+          <t>Tier 08 - Two Bedroom</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -5447,13 +5385,13 @@
         <v>2</v>
       </c>
       <c r="F44" s="5" t="n">
-        <v>990</v>
+        <v>982</v>
       </c>
       <c r="G44" s="6" t="n">
-        <v>4145</v>
+        <v>3993</v>
       </c>
       <c r="H44" s="6" t="n">
-        <v>4145</v>
+        <v>3993</v>
       </c>
       <c r="I44" s="7" t="n">
         <v>46113</v>
@@ -5466,7 +5404,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>1100-208</t>
+          <t>1100-408</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -5489,10 +5427,10 @@
         <v>982</v>
       </c>
       <c r="G45" s="6" t="n">
-        <v>3943</v>
+        <v>4018</v>
       </c>
       <c r="H45" s="6" t="n">
-        <v>3943</v>
+        <v>4018</v>
       </c>
       <c r="I45" s="7" t="n">
         <v>46113</v>
@@ -5505,7 +5443,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>1100-308</t>
+          <t>1100-508</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -5528,10 +5466,10 @@
         <v>982</v>
       </c>
       <c r="G46" s="6" t="n">
-        <v>3993</v>
+        <v>4043</v>
       </c>
       <c r="H46" s="6" t="n">
-        <v>3993</v>
+        <v>4043</v>
       </c>
       <c r="I46" s="7" t="n">
         <v>46113</v>
@@ -5544,7 +5482,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>1100-408</t>
+          <t>1100-608</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5567,10 +5505,10 @@
         <v>982</v>
       </c>
       <c r="G47" s="6" t="n">
-        <v>4018</v>
+        <v>4118</v>
       </c>
       <c r="H47" s="6" t="n">
-        <v>4018</v>
+        <v>4118</v>
       </c>
       <c r="I47" s="7" t="n">
         <v>46113</v>
@@ -5583,12 +5521,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>1100-508</t>
+          <t>1100-310</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Tier 08 - Two Bedroom</t>
+          <t>Tier 10 - Two Bedroom</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -5603,16 +5541,16 @@
         <v>2</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>982</v>
+        <v>934</v>
       </c>
       <c r="G48" s="6" t="n">
-        <v>4043</v>
+        <v>3745</v>
       </c>
       <c r="H48" s="6" t="n">
-        <v>4043</v>
+        <v>3745</v>
       </c>
       <c r="I48" s="7" t="n">
-        <v>46113</v>
+        <v>46094</v>
       </c>
       <c r="J48" s="8">
         <f>G48/F48</f>
@@ -5622,12 +5560,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>1100-608</t>
+          <t>1100-410</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Tier 08 - Two Bedroom</t>
+          <t>Tier 10 - Two Bedroom</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -5642,13 +5580,13 @@
         <v>2</v>
       </c>
       <c r="F49" s="5" t="n">
-        <v>982</v>
+        <v>934</v>
       </c>
       <c r="G49" s="6" t="n">
-        <v>4118</v>
+        <v>3820</v>
       </c>
       <c r="H49" s="6" t="n">
-        <v>4118</v>
+        <v>3820</v>
       </c>
       <c r="I49" s="7" t="n">
         <v>46113</v>
@@ -5661,7 +5599,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>1100-310</t>
+          <t>1100-610</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -5684,13 +5622,13 @@
         <v>934</v>
       </c>
       <c r="G50" s="6" t="n">
-        <v>3745</v>
+        <v>3920</v>
       </c>
       <c r="H50" s="6" t="n">
-        <v>3745</v>
+        <v>3920</v>
       </c>
       <c r="I50" s="7" t="n">
-        <v>46094</v>
+        <v>46113</v>
       </c>
       <c r="J50" s="8">
         <f>G50/F50</f>
@@ -5700,12 +5638,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>1100-410</t>
+          <t>1100-210</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Tier 10 - Two Bedroom</t>
+          <t>Tier 10 - Two Bedroom (Terrace)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -5723,10 +5661,10 @@
         <v>934</v>
       </c>
       <c r="G51" s="6" t="n">
-        <v>3820</v>
+        <v>4203</v>
       </c>
       <c r="H51" s="6" t="n">
-        <v>3820</v>
+        <v>4203</v>
       </c>
       <c r="I51" s="7" t="n">
         <v>46113</v>
@@ -5739,12 +5677,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>1100-610</t>
+          <t>1100-311</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Tier 10 - Two Bedroom</t>
+          <t>Tier 11 - Two Bedroom</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -5759,13 +5697,13 @@
         <v>2</v>
       </c>
       <c r="F52" s="5" t="n">
-        <v>934</v>
+        <v>972</v>
       </c>
       <c r="G52" s="6" t="n">
-        <v>3920</v>
+        <v>3898</v>
       </c>
       <c r="H52" s="6" t="n">
-        <v>3920</v>
+        <v>3898</v>
       </c>
       <c r="I52" s="7" t="n">
         <v>46113</v>
@@ -5778,12 +5716,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>1100-210</t>
+          <t>1100-411</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Tier 10 - Two Bedroom (Terrace)</t>
+          <t>Tier 11 - Two Bedroom</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -5798,13 +5736,13 @@
         <v>2</v>
       </c>
       <c r="F53" s="5" t="n">
-        <v>934</v>
+        <v>972</v>
       </c>
       <c r="G53" s="6" t="n">
-        <v>4203</v>
+        <v>3973</v>
       </c>
       <c r="H53" s="6" t="n">
-        <v>4203</v>
+        <v>3973</v>
       </c>
       <c r="I53" s="7" t="n">
         <v>46113</v>
@@ -5817,7 +5755,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>1100-311</t>
+          <t>1100-511</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -5840,10 +5778,10 @@
         <v>972</v>
       </c>
       <c r="G54" s="6" t="n">
-        <v>3898</v>
+        <v>3998</v>
       </c>
       <c r="H54" s="6" t="n">
-        <v>3898</v>
+        <v>3998</v>
       </c>
       <c r="I54" s="7" t="n">
         <v>46113</v>
@@ -5856,7 +5794,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>1100-411</t>
+          <t>1100-611</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -5876,13 +5814,13 @@
         <v>2</v>
       </c>
       <c r="F55" s="5" t="n">
-        <v>972</v>
+        <v>892</v>
       </c>
       <c r="G55" s="6" t="n">
-        <v>3973</v>
+        <v>3732</v>
       </c>
       <c r="H55" s="6" t="n">
-        <v>3973</v>
+        <v>3732</v>
       </c>
       <c r="I55" s="7" t="n">
         <v>46113</v>
@@ -5895,12 +5833,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>1100-511</t>
+          <t>1100-215</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Tier 11 - Two Bedroom</t>
+          <t>Tier 15 - Two Bedroom</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -5915,13 +5853,13 @@
         <v>2</v>
       </c>
       <c r="F56" s="5" t="n">
-        <v>972</v>
+        <v>1028</v>
       </c>
       <c r="G56" s="6" t="n">
-        <v>3998</v>
+        <v>4133</v>
       </c>
       <c r="H56" s="6" t="n">
-        <v>3998</v>
+        <v>4133</v>
       </c>
       <c r="I56" s="7" t="n">
         <v>46113</v>
@@ -5934,12 +5872,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>1100-611</t>
+          <t>1100-315</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Tier 11 - Two Bedroom</t>
+          <t>Tier 15 - Two Bedroom</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -5954,13 +5892,13 @@
         <v>2</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>892</v>
+        <v>1028</v>
       </c>
       <c r="G57" s="6" t="n">
-        <v>3732</v>
+        <v>4183</v>
       </c>
       <c r="H57" s="6" t="n">
-        <v>3732</v>
+        <v>4183</v>
       </c>
       <c r="I57" s="7" t="n">
         <v>46113</v>
@@ -5973,7 +5911,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>1100-215</t>
+          <t>1100-415</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -5996,10 +5934,10 @@
         <v>1028</v>
       </c>
       <c r="G58" s="6" t="n">
-        <v>4133</v>
+        <v>4233</v>
       </c>
       <c r="H58" s="6" t="n">
-        <v>4133</v>
+        <v>4233</v>
       </c>
       <c r="I58" s="7" t="n">
         <v>46113</v>
@@ -6012,7 +5950,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>1100-315</t>
+          <t>1100-515</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -6035,10 +5973,10 @@
         <v>1028</v>
       </c>
       <c r="G59" s="6" t="n">
-        <v>4183</v>
+        <v>4233</v>
       </c>
       <c r="H59" s="6" t="n">
-        <v>4183</v>
+        <v>4233</v>
       </c>
       <c r="I59" s="7" t="n">
         <v>46113</v>
@@ -6051,7 +5989,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>1100-415</t>
+          <t>1100-615</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -6074,10 +6012,10 @@
         <v>1028</v>
       </c>
       <c r="G60" s="6" t="n">
-        <v>4233</v>
+        <v>4308</v>
       </c>
       <c r="H60" s="6" t="n">
-        <v>4233</v>
+        <v>4308</v>
       </c>
       <c r="I60" s="7" t="n">
         <v>46113</v>
@@ -6090,12 +6028,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>1100-515</t>
+          <t>1100-217</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Tier 15 - Two Bedroom</t>
+          <t>Tier 17 - Two Bedroom</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -6110,13 +6048,13 @@
         <v>2</v>
       </c>
       <c r="F61" s="5" t="n">
-        <v>1028</v>
+        <v>917</v>
       </c>
       <c r="G61" s="6" t="n">
-        <v>4233</v>
+        <v>3495</v>
       </c>
       <c r="H61" s="6" t="n">
-        <v>4233</v>
+        <v>3495</v>
       </c>
       <c r="I61" s="7" t="n">
         <v>46113</v>
@@ -6129,12 +6067,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>1100-615</t>
+          <t>1100-317</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Tier 15 - Two Bedroom</t>
+          <t>Tier 17 - Two Bedroom</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -6149,13 +6087,13 @@
         <v>2</v>
       </c>
       <c r="F62" s="5" t="n">
-        <v>1028</v>
+        <v>917</v>
       </c>
       <c r="G62" s="6" t="n">
-        <v>4308</v>
+        <v>3721</v>
       </c>
       <c r="H62" s="6" t="n">
-        <v>4308</v>
+        <v>3721</v>
       </c>
       <c r="I62" s="7" t="n">
         <v>46113</v>
@@ -6168,7 +6106,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>1100-217</t>
+          <t>1100-517</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -6191,10 +6129,10 @@
         <v>917</v>
       </c>
       <c r="G63" s="6" t="n">
-        <v>3495</v>
+        <v>3771</v>
       </c>
       <c r="H63" s="6" t="n">
-        <v>3495</v>
+        <v>3771</v>
       </c>
       <c r="I63" s="7" t="n">
         <v>46113</v>
@@ -6207,7 +6145,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>1100-317</t>
+          <t>1100-617</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -6230,10 +6168,10 @@
         <v>917</v>
       </c>
       <c r="G64" s="6" t="n">
-        <v>3721</v>
+        <v>3846</v>
       </c>
       <c r="H64" s="6" t="n">
-        <v>3721</v>
+        <v>3846</v>
       </c>
       <c r="I64" s="7" t="n">
         <v>46113</v>
@@ -6246,33 +6184,33 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>1100-517</t>
+          <t>1100-307</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Tier 17 - Two Bedroom</t>
+          <t>Tier 07 - Three Bedroom</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2 Bedroom</t>
+          <t>3 Bedroom</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E65" t="n">
         <v>2</v>
       </c>
       <c r="F65" s="5" t="n">
-        <v>917</v>
+        <v>1166</v>
       </c>
       <c r="G65" s="6" t="n">
-        <v>3771</v>
+        <v>4964</v>
       </c>
       <c r="H65" s="6" t="n">
-        <v>3771</v>
+        <v>4964</v>
       </c>
       <c r="I65" s="7" t="n">
         <v>46113</v>
@@ -6285,33 +6223,33 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>1100-617</t>
+          <t>1100-407</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Tier 17 - Two Bedroom</t>
+          <t>Tier 07 - Three Bedroom</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2 Bedroom</t>
+          <t>3 Bedroom</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E66" t="n">
         <v>2</v>
       </c>
       <c r="F66" s="5" t="n">
-        <v>917</v>
+        <v>1166</v>
       </c>
       <c r="G66" s="6" t="n">
-        <v>3846</v>
+        <v>4989</v>
       </c>
       <c r="H66" s="6" t="n">
-        <v>3846</v>
+        <v>4989</v>
       </c>
       <c r="I66" s="7" t="n">
         <v>46113</v>
@@ -6324,7 +6262,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>1100-307</t>
+          <t>1100-507</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -6347,10 +6285,10 @@
         <v>1166</v>
       </c>
       <c r="G67" s="6" t="n">
-        <v>4964</v>
+        <v>5014</v>
       </c>
       <c r="H67" s="6" t="n">
-        <v>4964</v>
+        <v>5014</v>
       </c>
       <c r="I67" s="7" t="n">
         <v>46113</v>
@@ -6363,7 +6301,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>1100-407</t>
+          <t>1100-607</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -6386,10 +6324,10 @@
         <v>1166</v>
       </c>
       <c r="G68" s="6" t="n">
-        <v>4989</v>
+        <v>5089</v>
       </c>
       <c r="H68" s="6" t="n">
-        <v>4989</v>
+        <v>5089</v>
       </c>
       <c r="I68" s="7" t="n">
         <v>46113</v>
@@ -6402,12 +6340,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>1100-507</t>
+          <t>1100-719</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Tier 07 - Three Bedroom</t>
+          <t>Tier 19 - Penthouse</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -6422,13 +6360,13 @@
         <v>2</v>
       </c>
       <c r="F69" s="5" t="n">
-        <v>1166</v>
+        <v>1327</v>
       </c>
       <c r="G69" s="6" t="n">
-        <v>5014</v>
+        <v>6696</v>
       </c>
       <c r="H69" s="6" t="n">
-        <v>5014</v>
+        <v>6696</v>
       </c>
       <c r="I69" s="7" t="n">
         <v>46113</v>
@@ -6441,12 +6379,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>1100-607</t>
+          <t>1100-219</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Tier 07 - Three Bedroom</t>
+          <t>Tier 19 - Three Bedroom</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -6461,13 +6399,13 @@
         <v>2</v>
       </c>
       <c r="F70" s="5" t="n">
-        <v>1166</v>
+        <v>1327</v>
       </c>
       <c r="G70" s="6" t="n">
-        <v>5089</v>
+        <v>5582</v>
       </c>
       <c r="H70" s="6" t="n">
-        <v>5089</v>
+        <v>5582</v>
       </c>
       <c r="I70" s="7" t="n">
         <v>46113</v>
@@ -6480,12 +6418,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>1100-719</t>
+          <t>1100-319</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Tier 19 - Penthouse</t>
+          <t>Tier 19 - Three Bedroom</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -6503,10 +6441,10 @@
         <v>1327</v>
       </c>
       <c r="G71" s="6" t="n">
-        <v>6696</v>
+        <v>5607</v>
       </c>
       <c r="H71" s="6" t="n">
-        <v>6696</v>
+        <v>5607</v>
       </c>
       <c r="I71" s="7" t="n">
         <v>46113</v>
@@ -6519,7 +6457,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>1100-219</t>
+          <t>1100-419</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -6542,10 +6480,10 @@
         <v>1327</v>
       </c>
       <c r="G72" s="6" t="n">
-        <v>5582</v>
+        <v>5632</v>
       </c>
       <c r="H72" s="6" t="n">
-        <v>5582</v>
+        <v>5632</v>
       </c>
       <c r="I72" s="7" t="n">
         <v>46113</v>
@@ -6558,7 +6496,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>1100-319</t>
+          <t>1100-519</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -6581,10 +6519,10 @@
         <v>1327</v>
       </c>
       <c r="G73" s="6" t="n">
-        <v>5607</v>
+        <v>5657</v>
       </c>
       <c r="H73" s="6" t="n">
-        <v>5607</v>
+        <v>5657</v>
       </c>
       <c r="I73" s="7" t="n">
         <v>46113</v>
@@ -6597,7 +6535,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>1100-419</t>
+          <t>1100-619</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -6620,94 +6558,16 @@
         <v>1327</v>
       </c>
       <c r="G74" s="6" t="n">
-        <v>5632</v>
+        <v>5732</v>
       </c>
       <c r="H74" s="6" t="n">
-        <v>5632</v>
+        <v>5732</v>
       </c>
       <c r="I74" s="7" t="n">
         <v>46113</v>
       </c>
       <c r="J74" s="8">
         <f>G74/F74</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>1100-519</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>Tier 19 - Three Bedroom</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>3 Bedroom</t>
-        </is>
-      </c>
-      <c r="D75" t="n">
-        <v>3</v>
-      </c>
-      <c r="E75" t="n">
-        <v>2</v>
-      </c>
-      <c r="F75" s="5" t="n">
-        <v>1327</v>
-      </c>
-      <c r="G75" s="6" t="n">
-        <v>5657</v>
-      </c>
-      <c r="H75" s="6" t="n">
-        <v>5657</v>
-      </c>
-      <c r="I75" s="7" t="n">
-        <v>46113</v>
-      </c>
-      <c r="J75" s="8">
-        <f>G75/F75</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>1100-619</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>Tier 19 - Three Bedroom</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>3 Bedroom</t>
-        </is>
-      </c>
-      <c r="D76" t="n">
-        <v>3</v>
-      </c>
-      <c r="E76" t="n">
-        <v>2</v>
-      </c>
-      <c r="F76" s="5" t="n">
-        <v>1327</v>
-      </c>
-      <c r="G76" s="6" t="n">
-        <v>5732</v>
-      </c>
-      <c r="H76" s="6" t="n">
-        <v>5732</v>
-      </c>
-      <c r="I76" s="7" t="n">
-        <v>46113</v>
-      </c>
-      <c r="J76" s="8">
-        <f>G76/F76</f>
         <v/>
       </c>
     </row>

</xml_diff>